<commit_message>
Auto-atualização RTA - 18/09/2026 12:02
</commit_message>
<xml_diff>
--- a/downloads/RTA_Dados.xlsx
+++ b/downloads/RTA_Dados.xlsx
@@ -2720,7 +2720,7 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>Planejada</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -4041,7 +4041,7 @@
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
-          <t>Planejada</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">

</xml_diff>

<commit_message>
Auto-atualização RTA - 23/09/2026 12:02
</commit_message>
<xml_diff>
--- a/downloads/RTA_Dados.xlsx
+++ b/downloads/RTA_Dados.xlsx
@@ -10082,8 +10082,16 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="G160" t="inlineStr"/>
-      <c r="H160" t="inlineStr"/>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="I160" t="inlineStr">
         <is>
           <t>Causa: Falta de Planejamento na Execução da Atividade</t>
@@ -10097,10 +10105,14 @@
 A atividade foi inicialmente planejada para substituição da junta do Multijato do Cozedor 01, devido a vazamento identificado durante a operação. No decorrer da execução, foram identificadas falhas adicionais na válvula e problemas estruturais na tubulação, ampliando o escopo da manutenção.</t>
         </is>
       </c>
-      <c r="K160" t="inlineStr"/>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>Válvulas validadas no plano de Entressafra</t>
+        </is>
+      </c>
       <c r="L160" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M160" t="inlineStr">
@@ -10198,8 +10210,16 @@
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="G162" t="inlineStr"/>
-      <c r="H162" t="inlineStr"/>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="I162" t="inlineStr">
         <is>
           <t>Causa: Falta de Planejamento na Execução da Atividade</t>
@@ -10213,10 +10233,14 @@
 A atividade foi inicialmente planejada para substituição da junta do Multijato do Cozedor 01, devido a vazamento identificado durante a operação. No decorrer da execução, foram identificadas falhas adicionais na válvula e problemas estruturais na tubulação, ampliando o escopo da manutenção.</t>
         </is>
       </c>
-      <c r="K162" t="inlineStr"/>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>foi implementado reuniões diversas de parada por chuva e semanal</t>
+        </is>
+      </c>
       <c r="L162" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M162" t="inlineStr">
@@ -12662,8 +12686,16 @@
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="G199" t="inlineStr"/>
-      <c r="H199" t="inlineStr"/>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="I199" t="inlineStr">
         <is>
           <t>Causa: Impressão da programação/falha de comunicação</t>
@@ -12676,10 +12708,15 @@
 Frentes abertas sem alinhamento entre as áreas.</t>
         </is>
       </c>
-      <c r="K199" t="inlineStr"/>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>Sendo executado semanalmente.
+Sendo enviado nos grupos</t>
+        </is>
+      </c>
       <c r="L199" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M199" t="inlineStr">
@@ -12719,8 +12756,16 @@
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="G200" t="inlineStr"/>
-      <c r="H200" t="inlineStr"/>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="I200" t="inlineStr">
         <is>
           <t>Causa: Impressão da programação/falha de comunicação</t>
@@ -12733,10 +12778,14 @@
 Frentes abertas sem alinhamento entre as áreas.</t>
         </is>
       </c>
-      <c r="K200" t="inlineStr"/>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>Só é seguido o que está nas listas divulgadas</t>
+        </is>
+      </c>
       <c r="L200" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M200" t="inlineStr">
@@ -12776,8 +12825,16 @@
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="G201" t="inlineStr"/>
-      <c r="H201" t="inlineStr"/>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="I201" t="inlineStr">
         <is>
           <t>Causa: Impressão da programação/falha de comunicação</t>
@@ -12790,10 +12847,14 @@
 Frentes abertas sem alinhamento entre as áreas.</t>
         </is>
       </c>
-      <c r="K201" t="inlineStr"/>
+      <c r="K201" t="inlineStr">
+        <is>
+          <t>Programação semanal executada toda quinta</t>
+        </is>
+      </c>
       <c r="L201" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M201" t="inlineStr">
@@ -12833,8 +12894,16 @@
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="G202" t="inlineStr"/>
-      <c r="H202" t="inlineStr"/>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="I202" t="inlineStr">
         <is>
           <t>Causa: Impressão de programação/falha de comunicação</t>
@@ -12847,10 +12916,14 @@
 Frentes abertas sem alinhamento entre as áreas.</t>
         </is>
       </c>
-      <c r="K202" t="inlineStr"/>
+      <c r="K202" t="inlineStr">
+        <is>
+          <t>Programação enviada para todo plantonista no GRUPO de PCM</t>
+        </is>
+      </c>
       <c r="L202" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M202" t="inlineStr">
@@ -13022,8 +13095,16 @@
           <t>2026-05-29</t>
         </is>
       </c>
-      <c r="G205" t="inlineStr"/>
-      <c r="H205" t="inlineStr"/>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="I205" t="inlineStr">
         <is>
           <t>Causa: Falta de Formalização do Plano de Manutenção</t>
@@ -13034,10 +13115,14 @@
           <t>Trip da Turbina do segundo terno, após a turbina rodava em campo mas não indicava no COI</t>
         </is>
       </c>
-      <c r="K205" t="inlineStr"/>
+      <c r="K205" t="inlineStr">
+        <is>
+          <t>Inspeção sendo realizada</t>
+        </is>
+      </c>
       <c r="L205" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M205" t="inlineStr">
@@ -14628,8 +14713,16 @@
           <t>2026-07-15</t>
         </is>
       </c>
-      <c r="G229" t="inlineStr"/>
-      <c r="H229" t="inlineStr"/>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="I229" t="inlineStr">
         <is>
           <t>Causa: Baixa qualidade do eletrodo de solda</t>
@@ -14644,10 +14737,15 @@
 3) Instalação de novo pente de saída;</t>
         </is>
       </c>
-      <c r="K229" t="inlineStr"/>
+      <c r="K229" t="inlineStr">
+        <is>
+          <t>Tema finalizado
+Saldo não liberado</t>
+        </is>
+      </c>
       <c r="L229" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M229" t="inlineStr">
@@ -14687,8 +14785,16 @@
           <t>2026-07-31</t>
         </is>
       </c>
-      <c r="G230" t="inlineStr"/>
-      <c r="H230" t="inlineStr"/>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="I230" t="inlineStr">
         <is>
           <t>Causa: Baixa qualidade do eletrodo de solda</t>
@@ -14703,10 +14809,14 @@
 3) Instalação de novo pente de saída;</t>
         </is>
       </c>
-      <c r="K230" t="inlineStr"/>
+      <c r="K230" t="inlineStr">
+        <is>
+          <t>Item OK</t>
+        </is>
+      </c>
       <c r="L230" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M230" t="inlineStr">
@@ -14746,8 +14856,16 @@
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="G231" t="inlineStr"/>
-      <c r="H231" t="inlineStr"/>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="I231" t="inlineStr">
         <is>
           <t>Causa: Baixa qualidade do eletrodo de solda</t>
@@ -14762,10 +14880,15 @@
 3) Instalação de novo pente de saída;</t>
         </is>
       </c>
-      <c r="K231" t="inlineStr"/>
+      <c r="K231" t="inlineStr">
+        <is>
+          <t>Item OK.
+Material devidamente cadastrado</t>
+        </is>
+      </c>
       <c r="L231" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M231" t="inlineStr">

</xml_diff>

<commit_message>
Auto-atualização RTA - 23/09/2026 14:38
</commit_message>
<xml_diff>
--- a/downloads/RTA_Dados.xlsx
+++ b/downloads/RTA_Dados.xlsx
@@ -4265,8 +4265,16 @@
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="G67" t="inlineStr"/>
-      <c r="H67" t="inlineStr"/>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
       <c r="I67" t="inlineStr">
         <is>
           <t>Causa: Proteção Ineficiente</t>
@@ -4277,10 +4285,14 @@
           <t>Trip do Turbo-gerador  por acionamento indevido da botoeira de emergência Geral</t>
         </is>
       </c>
-      <c r="K67" t="inlineStr"/>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Foi realizado proteção dos emergência da sala operacional do turbo gerador, fotos estão em anexo </t>
+        </is>
+      </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>Planejada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
@@ -4454,8 +4466,16 @@
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr"/>
-      <c r="H70" t="inlineStr"/>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
       <c r="I70" t="inlineStr">
         <is>
           <t>Causa: Acionamento indevido do botão de emergência</t>
@@ -4466,10 +4486,14 @@
           <t>Trip do Turbo-gerador  por acionamento indevido da botoeira de emergência Geral</t>
         </is>
       </c>
-      <c r="K70" t="inlineStr"/>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>Plano finalizado. Foram retiradas todas as cadeiras da sala operacional, permanecendo somente a cadeira destinada ao operador, conforme solicitado no plano de ação.</t>
+        </is>
+      </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
@@ -5451,8 +5475,16 @@
           <t>2026-07-31</t>
         </is>
       </c>
-      <c r="G87" t="inlineStr"/>
-      <c r="H87" t="inlineStr"/>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
       <c r="I87" t="inlineStr">
         <is>
           <t>Causa: Porque houve quebra da correia da bomba de cal</t>
@@ -5465,10 +5497,14 @@
 No dia 18/07, houve a quebra da correia da bomba de cal. Além disso, verificou-se que a bomba não estava eficiente, então, foi realizada a substituição da bomba.</t>
         </is>
       </c>
-      <c r="K87" t="inlineStr"/>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Foi substituida as correias das bombas de cal </t>
+        </is>
+      </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M87" t="inlineStr">
@@ -13162,8 +13198,16 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="G206" t="inlineStr"/>
-      <c r="H206" t="inlineStr"/>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
       <c r="I206" t="inlineStr">
         <is>
           <t>Causa: Falta de Formalização do Plano de Manutenção</t>
@@ -13174,10 +13218,14 @@
           <t>Trip da Turbina do segundo terno, após a turbina rodava em campo mas não indicava no COI</t>
         </is>
       </c>
-      <c r="K206" t="inlineStr"/>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>Foi realizado a inspeção nos pick-up das turbinas durante a parada. Ordem de serviço 57666.</t>
+        </is>
+      </c>
       <c r="L206" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M206" t="inlineStr">
@@ -13272,8 +13320,16 @@
           <t>2026-05-29</t>
         </is>
       </c>
-      <c r="G208" t="inlineStr"/>
-      <c r="H208" t="inlineStr"/>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
       <c r="I208" t="inlineStr">
         <is>
           <t>Causa: Falta de conhecimento sobre o componente mecânico</t>
@@ -13284,10 +13340,14 @@
           <t>Trip da Turbina do segundo terno, após a turbina rodava em campo mas não indicava no COI</t>
         </is>
       </c>
-      <c r="K208" t="inlineStr"/>
+      <c r="K208" t="inlineStr">
+        <is>
+          <t>Foi feito treinamento com os eletricistas dos turnos sobre o funcionamento do indicador de RPM das turbinas, deixando os mesmos aptos para identificar defeitos no mesmo ou problemas mecânicos que possam interferir na indicação de RPM.</t>
+        </is>
+      </c>
       <c r="L208" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M208" t="inlineStr">
@@ -29925,7 +29985,7 @@
       </c>
       <c r="H463" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="I463" t="inlineStr">

</xml_diff>

<commit_message>
Auto-atualização RTA - 25/09/2026 12:02
</commit_message>
<xml_diff>
--- a/downloads/RTA_Dados.xlsx
+++ b/downloads/RTA_Dados.xlsx
@@ -867,7 +867,7 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Planejada</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -924,7 +924,7 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Planejada</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1286,7 +1286,7 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>Atrasada</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2229,7 +2229,7 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
-          <t>Planejada</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2343,7 +2343,7 @@
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Planejada</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -3594,7 +3594,7 @@
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>Atrasada</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
@@ -5435,7 +5435,7 @@
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
-          <t>Planejada</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="M86" t="inlineStr">
@@ -6219,7 +6219,7 @@
       <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr">
         <is>
-          <t>Planejada</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="M99" t="inlineStr">

</xml_diff>

<commit_message>
Auto-atualização RTA - 26/09/2026 12:02
</commit_message>
<xml_diff>
--- a/downloads/RTA_Dados.xlsx
+++ b/downloads/RTA_Dados.xlsx
@@ -867,7 +867,7 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>Atrasada</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -924,7 +924,7 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>Atrasada</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -2229,7 +2229,7 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>Atrasada</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2343,7 +2343,7 @@
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>Atrasada</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -3207,8 +3207,16 @@
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr"/>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
       <c r="I49" t="inlineStr">
         <is>
           <t>Causa: Elevado tempo entre as coletas pelo amostrador</t>
@@ -3226,10 +3234,14 @@
 [fig:vfs:2854]</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr"/>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Conforme  solicitado, foram ajustados tempos de coletas simultâneas entrada e retorno da agua Spray</t>
+        </is>
+      </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
@@ -3269,8 +3281,16 @@
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr"/>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
       <c r="I50" t="inlineStr">
         <is>
           <t>Causa: Elevado tempo entre as coletas pelo amostrador</t>
@@ -3288,10 +3308,14 @@
 [fig:vfs:2854]</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr"/>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Ficou definido que a amostragem será realizada automaticamente a cada 5 minutos pelo amostrador, formando uma amostra composta. A cada 4 horas, essa amostra será coletada pelo técnico, armazenada no congelador do laboratório e analisada durante o turno da noite.</t>
+        </is>
+      </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
@@ -3331,8 +3355,16 @@
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
       <c r="I51" t="inlineStr">
         <is>
           <t>Causa: Desvio na execução da análise</t>
@@ -3350,10 +3382,14 @@
 [fig:vfs:2854]</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr"/>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Foi acompanhado os técnicos em suas atividades e não encontrados desvios na realização das analises </t>
+        </is>
+      </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
@@ -3517,8 +3553,16 @@
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
       <c r="I54" t="inlineStr">
         <is>
           <t>Causa: Baixa frequência de análise</t>
@@ -3536,10 +3580,14 @@
 [fig:vfs:2854]</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr"/>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>O plano analítico foi definido no início do ano, antes do começo da safra, com o alinhamento e concordância dos supervisores. Ficou estabelecido que as análises seriam realizadas uma vez ao dia. Caso ocorra alguma perda ou desvio no processo, deverá ser aberta uma exceção para aumentar a frequência das análises nos demais turnos até que a situação seja normalizada.</t>
+        </is>
+      </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
@@ -5435,7 +5483,7 @@
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>Atrasada</t>
         </is>
       </c>
       <c r="M86" t="inlineStr">
@@ -6219,7 +6267,7 @@
       <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>Atrasada</t>
         </is>
       </c>
       <c r="M99" t="inlineStr">
@@ -11407,8 +11455,16 @@
           <t>2026-06-05</t>
         </is>
       </c>
-      <c r="G179" t="inlineStr"/>
-      <c r="H179" t="inlineStr"/>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
       <c r="I179" t="inlineStr">
         <is>
           <t>Causa: Por que o aparelho é novo e ainda esta em fase de testes</t>
@@ -11422,10 +11478,14 @@
 Em alinhamento com o laboratório ficou definido que: quando houver uma parada de aparelho, a média de perdas deverá ser ponderada pela produção do último horário de cada aparelho, o que garante que a análise seja registrada mas a perda contemple apenas o período de produção.</t>
         </is>
       </c>
-      <c r="K179" t="inlineStr"/>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>Procedimento alinhado com a Supervisora da Destilaria e validado. A ação será feita em conjunto com o laboratório para garantir imparcialidade.</t>
+        </is>
+      </c>
       <c r="L179" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M179" t="inlineStr">
@@ -12026,8 +12086,16 @@
           <t>2026-05-22</t>
         </is>
       </c>
-      <c r="G188" t="inlineStr"/>
-      <c r="H188" t="inlineStr"/>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
       <c r="I188" t="inlineStr">
         <is>
           <t>Causa: Dificuldade na tomada decisão na alimentação e controle fermentativo</t>
@@ -12038,10 +12106,14 @@
           <t>Baixa eficiência devido complicações com alta contaminação, e dificuldade na mensuração de ARRT da última dorna causado pela instabilidade do cromatógrafo.</t>
         </is>
       </c>
-      <c r="K188" t="inlineStr"/>
+      <c r="K188" t="inlineStr">
+        <is>
+          <t>Ação não foi feita em conjunto e não entendi o que foi solicitado. Que metodologia? Qual análise? Qual amostra?</t>
+        </is>
+      </c>
       <c r="L188" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M188" t="inlineStr">
@@ -14054,8 +14126,16 @@
           <t>2026-06-08</t>
         </is>
       </c>
-      <c r="G218" t="inlineStr"/>
-      <c r="H218" t="inlineStr"/>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
       <c r="I218" t="inlineStr">
         <is>
           <t>Causa: Por que houve uma passagem de matéria prima ruim</t>
@@ -14072,10 +14152,14 @@
 [fig:vfs:2449]</t>
         </is>
       </c>
-      <c r="K218" t="inlineStr"/>
+      <c r="K218" t="inlineStr">
+        <is>
+          <t>Manutenção concluída e instado no local,  realizado configuração comissionado e colocado em operação.</t>
+        </is>
+      </c>
       <c r="L218" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M218" t="inlineStr">
@@ -14188,8 +14272,16 @@
           <t>2026-05-29</t>
         </is>
       </c>
-      <c r="G220" t="inlineStr"/>
-      <c r="H220" t="inlineStr"/>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
       <c r="I220" t="inlineStr">
         <is>
           <t>Causa: Por que houve uma passagem de matéria prima ruim</t>
@@ -14206,10 +14298,14 @@
 [fig:vfs:2449]</t>
         </is>
       </c>
-      <c r="K220" t="inlineStr"/>
+      <c r="K220" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Realizado o alinhamento com Cristiano do COA para realizar o Blender nas mesas de cana </t>
+        </is>
+      </c>
       <c r="L220" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M220" t="inlineStr">
@@ -18962,8 +19058,16 @@
           <t>2025-12-15</t>
         </is>
       </c>
-      <c r="G292" t="inlineStr"/>
-      <c r="H292" t="inlineStr"/>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
       <c r="I292" t="inlineStr">
         <is>
           <t>Causa: Não chegando na pureza necessária da cana</t>
@@ -18974,10 +19078,14 @@
           <t>Em novembro possivelmente iniciou a entrada de cana do cana com impureza, impactando assim a eficiência e pureza da massa A e B da usina</t>
         </is>
       </c>
-      <c r="K292" t="inlineStr"/>
+      <c r="K292" t="inlineStr">
+        <is>
+          <t>Isso já foi definido e está na plano de análise.</t>
+        </is>
+      </c>
       <c r="L292" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M292" t="inlineStr">
@@ -20339,7 +20447,7 @@
       </c>
       <c r="F314" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2027-12-08</t>
         </is>
       </c>
       <c r="G314" t="inlineStr"/>
@@ -20571,7 +20679,7 @@
       </c>
       <c r="F318" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2027-12-08</t>
         </is>
       </c>
       <c r="G318" t="inlineStr"/>

</xml_diff>

<commit_message>
Auto-atualização RTA - 02/10/2026 12:02
</commit_message>
<xml_diff>
--- a/downloads/RTA_Dados.xlsx
+++ b/downloads/RTA_Dados.xlsx
@@ -1036,7 +1036,7 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Planejada</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1091,7 +1091,7 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Planejada</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -7734,8 +7734,16 @@
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="G121" t="inlineStr"/>
-      <c r="H121" t="inlineStr"/>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
       <c r="I121" t="inlineStr">
         <is>
           <t>Causa: teste</t>
@@ -7749,7 +7757,7 @@
       <c r="K121" t="inlineStr"/>
       <c r="L121" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M121" t="inlineStr">
@@ -10457,8 +10465,16 @@
           <t>2026-07-31</t>
         </is>
       </c>
-      <c r="G163" t="inlineStr"/>
-      <c r="H163" t="inlineStr"/>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="I163" t="inlineStr">
         <is>
           <t>Causa: Falta de Planejamento na Execução da Atividade</t>
@@ -10472,10 +10488,15 @@
 A atividade foi inicialmente planejada para substituição da junta do Multijato do Cozedor 01, devido a vazamento identificado durante a operação. No decorrer da execução, foram identificadas falhas adicionais na válvula e problemas estruturais na tubulação, ampliando o escopo da manutenção.</t>
         </is>
       </c>
-      <c r="K163" t="inlineStr"/>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>Segue levantamento que a manutenção da instrumentação realizou juntamente com o time da Fabrica, ja tinha sido finalizado a ação porem não estava conseguindo lançar a evidencia
+[fig:vfs:3214]</t>
+        </is>
+      </c>
       <c r="L163" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M163" t="inlineStr">
@@ -10713,8 +10734,16 @@
           <t>2026-07-31</t>
         </is>
       </c>
-      <c r="G167" t="inlineStr"/>
-      <c r="H167" t="inlineStr"/>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="I167" t="inlineStr">
         <is>
           <t>Causa: Falta de Planejamento de Execução da Atividade</t>
@@ -10728,10 +10757,16 @@
 A atividade foi inicialmente planejada para substituição da junta do Multijato do Cozedor 01, devido a vazamento identificado durante a operação. No decorrer da execução, foram identificadas falhas adicionais na válvula e problemas estruturais na tubulação, ampliando o escopo da manutenção.</t>
         </is>
       </c>
-      <c r="K167" t="inlineStr"/>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Foi alinhado com os lideres e adicionado na ATA do dia 28/07 do RITO da Fábrica.
+[fig:vfs:3215]
+</t>
+        </is>
+      </c>
       <c r="L167" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M167" t="inlineStr">

</xml_diff>

<commit_message>
Auto-atualização RTA - 03/10/2026 12:02
</commit_message>
<xml_diff>
--- a/downloads/RTA_Dados.xlsx
+++ b/downloads/RTA_Dados.xlsx
@@ -1036,7 +1036,7 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>Atrasada</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1091,7 +1091,7 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>Atrasada</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">

</xml_diff>

<commit_message>
Auto-atualização RTA - 05/10/2026 19:02
</commit_message>
<xml_diff>
--- a/downloads/RTA_Dados.xlsx
+++ b/downloads/RTA_Dados.xlsx
@@ -1546,8 +1546,16 @@
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
       <c r="I20" t="inlineStr">
         <is>
           <t>Causa: Falta de Ferramental adequado para atividade</t>
@@ -1558,10 +1566,14 @@
           <t>Durante a parada da Caldeira 3 foi decidido retirar o By pass</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr"/>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Empresa Homologada, processo em andamento de contratação</t>
+        </is>
+      </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -1986,8 +1998,16 @@
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
       <c r="I28" t="inlineStr">
         <is>
           <t>Causa: Mapeamento executado dentro da priorzação da Entressafra 25/26</t>
@@ -1998,10 +2018,14 @@
           <t>Vazamento no Superaquecedor que foi detectado ao longo do dia, em alinhamento com a liderança iríamos manter o processo até fechar o dia porém, vazamento ampliou, havendo necessidade de realizar a intervenção após o resfriamento.</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr"/>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Reunião de planejamento em execução de forma fixa e conforme necessidade</t>
+        </is>
+      </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -4905,8 +4929,16 @@
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr"/>
-      <c r="H76" t="inlineStr"/>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
       <c r="I76" t="inlineStr">
         <is>
           <t>Causa: Falta de detecção de vibração</t>
@@ -4918,10 +4950,15 @@
 Ocorreu avaria do conjunto rotativo, causando danos no eixo principal e no espaçador, o que resultou na parada não programada do equipamento. Na inspeção realizada, foram observados desgaste acentuado e marcas de atrito, deformações na superfície e a fratura do espaçador, indicando que o conjunto perdeu sua integridade mecânica.</t>
         </is>
       </c>
-      <c r="K76" t="inlineStr"/>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>Estou encerrando a ação.
+Não temos saldo para fazer isso, fizemos um levantamento geral de todos os pontos críticos, foi apresentado ao gerente, mas não seguiremos por ora.</t>
+        </is>
+      </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M76" t="inlineStr">
@@ -10606,8 +10643,16 @@
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="G165" t="inlineStr"/>
-      <c r="H165" t="inlineStr"/>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
       <c r="I165" t="inlineStr">
         <is>
           <t>Causa: Falta de Planejamento na execução da atividade</t>
@@ -10621,10 +10666,15 @@
 A atividade foi inicialmente planejada para substituição da junta do Multijato do Cozedor 01, devido a vazamento identificado durante a operação. No decorrer da execução, foram identificadas falhas adicionais na válvula e problemas estruturais na tubulação, ampliando o escopo da manutenção.</t>
         </is>
       </c>
-      <c r="K165" t="inlineStr"/>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>Bom Dia!
+Valvulas corretamente especificadas</t>
+        </is>
+      </c>
       <c r="L165" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M165" t="inlineStr">
@@ -13721,8 +13771,16 @@
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="G211" t="inlineStr"/>
-      <c r="H211" t="inlineStr"/>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
       <c r="I211" t="inlineStr">
         <is>
           <t>Causa: Falta de Formalização do Plano de Manutenção</t>
@@ -13733,10 +13791,14 @@
           <t>Trip da Turbina do segundo terno, após a turbina rodava em campo mas não indicava no COI</t>
         </is>
       </c>
-      <c r="K211" t="inlineStr"/>
+      <c r="K211" t="inlineStr">
+        <is>
+          <t>Máscara padrão criada</t>
+        </is>
+      </c>
       <c r="L211" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M211" t="inlineStr">

</xml_diff>

<commit_message>
Auto-atualização RTA - 07/10/2026 12:02
</commit_message>
<xml_diff>
--- a/downloads/RTA_Dados.xlsx
+++ b/downloads/RTA_Dados.xlsx
@@ -1491,8 +1491,16 @@
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr">
         <is>
           <t>Causa: Arraste no aspersor</t>
@@ -1503,10 +1511,14 @@
           <t>No dia 17/08 no turno A tivemos uma ocorrência de arraste no aspersor</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr"/>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Realizado inspeção rotineira pelo Operador de evaporação 2 vezes por turno para acompanhamento das perdas</t>
+        </is>
+      </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -3919,8 +3931,16 @@
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
       <c r="I59" t="inlineStr">
         <is>
           <t>Causa: rwer</t>
@@ -3932,7 +3952,7 @@
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
@@ -4873,8 +4893,16 @@
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr"/>
-      <c r="H75" t="inlineStr"/>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
       <c r="I75" t="inlineStr">
         <is>
           <t>Causa: Falha na rotina de limpeza</t>
@@ -4886,10 +4914,15 @@
 Ocorreu avaria do conjunto rotativo, causando danos no eixo principal e no espaçador, o que resultou na parada não programada do equipamento. Na inspeção realizada, foram observados desgaste acentuado e marcas de atrito, deformações na superfície e a fratura do espaçador, indicando que o conjunto perdeu sua integridade mecânica.</t>
         </is>
       </c>
-      <c r="K75" t="inlineStr"/>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>Avaliado rotina de limpeza operacional das konts.
+As Konts já possuem sistema de limpeza automatico a cada 8 horas onde a maquina para a sua operação para efetuar a limpeza da tela.</t>
+        </is>
+      </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M75" t="inlineStr">
@@ -6181,8 +6214,16 @@
           <t>2026-07-20</t>
         </is>
       </c>
-      <c r="G96" t="inlineStr"/>
-      <c r="H96" t="inlineStr"/>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
       <c r="I96" t="inlineStr">
         <is>
           <t>Causa: TESTE</t>
@@ -6196,7 +6237,7 @@
       <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M96" t="inlineStr">
@@ -7834,8 +7875,16 @@
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="G122" t="inlineStr"/>
-      <c r="H122" t="inlineStr"/>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
       <c r="I122" t="inlineStr">
         <is>
           <t>Causa: teste</t>
@@ -7849,7 +7898,7 @@
       <c r="K122" t="inlineStr"/>
       <c r="L122" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M122" t="inlineStr">
@@ -7904,7 +7953,7 @@
       <c r="K123" t="inlineStr"/>
       <c r="L123" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Suspensa</t>
         </is>
       </c>
       <c r="M123" t="inlineStr">
@@ -8302,8 +8351,16 @@
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="G130" t="inlineStr"/>
-      <c r="H130" t="inlineStr"/>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
       <c r="I130" t="inlineStr">
         <is>
           <t>Causa: dasd</t>
@@ -8317,7 +8374,7 @@
       <c r="K130" t="inlineStr"/>
       <c r="L130" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M130" t="inlineStr">
@@ -9314,7 +9371,11 @@
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="H146" t="inlineStr"/>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
       <c r="I146" t="inlineStr">
         <is>
           <t>Causa: Dificuldade de controle na concentração de lodo</t>
@@ -9336,10 +9397,15 @@
 - Problemas com ajustes operacionais</t>
         </is>
       </c>
-      <c r="K146" t="inlineStr"/>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+[fig:vfs:3250]</t>
+        </is>
+      </c>
       <c r="L146" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M146" t="inlineStr">
@@ -10444,8 +10510,16 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="G162" t="inlineStr"/>
-      <c r="H162" t="inlineStr"/>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
       <c r="I162" t="inlineStr">
         <is>
           <t>Causa: Falta de Planejamento na execução da atividade</t>
@@ -10459,10 +10533,19 @@
 A atividade foi inicialmente planejada para substituição da junta do Multijato do Cozedor 01, devido a vazamento identificado durante a operação. No decorrer da execução, foram identificadas falhas adicionais na válvula e problemas estruturais na tubulação, ampliando o escopo da manutenção.</t>
         </is>
       </c>
-      <c r="K162" t="inlineStr"/>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Os multijatos adquiridos não foram fornecidos com juntas de vedação. Dessa forma, foram instalados sem as referidas juntas, o que ocasionou vazamentos durante a operação. Posteriormente, as juntas de vedação foram instaladas e, atualmente, os multijatos operam normalmente, sem ocorrência de vazamentos.
+Quanto à tubulação de vapor de saída do Cozedor 1, ocorreu uma falha por implosão, ocasionando o colapso de um trecho da tubulação. Na ocasião, o trecho danificado foi substituído por uma tubulação de diâmetro inferior ao original, condição que permanece atualmente.
+Não foi realizada inspeção no trecho localizado a montante do ponto de colapso. Entretanto, foi realizada inspeção de espessura no trecho a jusante, sendo constatada espessura dentro dos parâmetros considerados regulares.
+As inspeções dos equipamentos são realizadas pelo time de Confiabilidade. As recomposições decorrentes de desgastes e demais intervenções de manutenção são realizadas pelo time de Manutenção.
+Até o momento, não foi identificada a necessidade de elaboração de projeto. Caso seja identificada alguma necessidade nesse sentido, favor entrar em contato.
+</t>
+        </is>
+      </c>
       <c r="L162" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M162" t="inlineStr">
@@ -12978,8 +13061,16 @@
           <t>2027-03-01</t>
         </is>
       </c>
-      <c r="G199" t="inlineStr"/>
-      <c r="H199" t="inlineStr"/>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
       <c r="I199" t="inlineStr">
         <is>
           <t>Causa: Porque não foi feito manutenção preventiva no separador</t>
@@ -13000,10 +13091,14 @@
 [fig:vfs:2465]</t>
         </is>
       </c>
-      <c r="K199" t="inlineStr"/>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>Realizado a instalação das chapas defletoras pela equipe de caldeiraria</t>
+        </is>
+      </c>
       <c r="L199" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M199" t="inlineStr">
@@ -14462,8 +14557,16 @@
           <t>2026-05-22</t>
         </is>
       </c>
-      <c r="G220" t="inlineStr"/>
-      <c r="H220" t="inlineStr"/>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
       <c r="I220" t="inlineStr">
         <is>
           <t>Causa: Por conta das passantes muito alta e assoreamento na área e alguns pontos com excesso de umidade</t>
@@ -14474,10 +14577,16 @@
           <t>Dos dias 01 ao dia 06 de maio não conseguiu atingir a meta de eficiência operacional no plantio frente 2.</t>
         </is>
       </c>
-      <c r="K220" t="inlineStr"/>
+      <c r="K220" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Plano de ação concluído, equipe de qualidade agrícola iniciou a realização de avaliação de qualidade de sistematização.
+[fig:vfs:3246]</t>
+        </is>
+      </c>
       <c r="L220" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M220" t="inlineStr">

</xml_diff>

<commit_message>
Auto-atualização RTA - 09/10/2026 12:02
</commit_message>
<xml_diff>
--- a/downloads/RTA_Dados.xlsx
+++ b/downloads/RTA_Dados.xlsx
@@ -754,7 +754,7 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Planejada</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -810,7 +810,7 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Planejada</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1146,7 +1146,7 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Planejada</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">

</xml_diff>

<commit_message>
Auto-atualização RTA - 14/10/2026 12:02
</commit_message>
<xml_diff>
--- a/downloads/RTA_Dados.xlsx
+++ b/downloads/RTA_Dados.xlsx
@@ -5668,7 +5668,7 @@
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
-          <t>Planejada</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="M87" t="inlineStr">
@@ -8340,8 +8340,16 @@
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="G130" t="inlineStr"/>
-      <c r="H130" t="inlineStr"/>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
       <c r="I130" t="inlineStr">
         <is>
           <t>Causa: Mudanç de área</t>
@@ -8352,10 +8360,14 @@
           <t>Frente 25 não atingiu a eficiência operacional por mudança de área</t>
         </is>
       </c>
-      <c r="K130" t="inlineStr"/>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>Realizado</t>
+        </is>
+      </c>
       <c r="L130" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M130" t="inlineStr">
@@ -8395,8 +8407,16 @@
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="G131" t="inlineStr"/>
-      <c r="H131" t="inlineStr"/>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
       <c r="I131" t="inlineStr">
         <is>
           <t>Causa: Ponte - Faz Santa Barbara</t>
@@ -8407,10 +8427,14 @@
           <t>A frente 25 ficou fora da eficiência motor com o maior ofensor turno por mudança de área</t>
         </is>
       </c>
-      <c r="K131" t="inlineStr"/>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>Realizado</t>
+        </is>
+      </c>
       <c r="L131" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M131" t="inlineStr">

</xml_diff>

<commit_message>
Auto-atualização RTA - 15/10/2026 12:02
</commit_message>
<xml_diff>
--- a/downloads/RTA_Dados.xlsx
+++ b/downloads/RTA_Dados.xlsx
@@ -1560,7 +1560,7 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Planejada</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -5668,7 +5668,7 @@
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>Atrasada</t>
         </is>
       </c>
       <c r="M87" t="inlineStr">

</xml_diff>

<commit_message>
Auto-atualização RTA - 16/10/2026 12:02
</commit_message>
<xml_diff>
--- a/downloads/RTA_Dados.xlsx
+++ b/downloads/RTA_Dados.xlsx
@@ -1434,7 +1434,7 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Planejada</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1560,7 +1560,7 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>Atrasada</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2653,7 +2653,7 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>Planejada</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">

</xml_diff>

<commit_message>
Auto-atualização RTA - 17/10/2026 12:02
</commit_message>
<xml_diff>
--- a/downloads/RTA_Dados.xlsx
+++ b/downloads/RTA_Dados.xlsx
@@ -1434,7 +1434,7 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>Atrasada</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2653,7 +2653,7 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>Atrasada</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">

</xml_diff>

<commit_message>
Auto-atualização RTA - 23/10/2026 12:02
</commit_message>
<xml_diff>
--- a/downloads/RTA_Dados.xlsx
+++ b/downloads/RTA_Dados.xlsx
@@ -529,7 +529,7 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Planejada</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -640,7 +640,7 @@
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>Atrasada</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -680,8 +680,16 @@
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
           <t>Causa: falta conscientização do colaborador para realizar a os apontamentos</t>
@@ -692,10 +700,15 @@
           <t>Das 171 frotas programadas para as semanas 40/41 11% ficou sem justificativa e 23,4% ficou sem apontamento.</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Feito
+</t>
+        </is>
+      </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -735,8 +748,16 @@
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr">
         <is>
           <t>Causa: falta conscientização do colaborador para realizar a os apontamentos</t>
@@ -747,10 +768,15 @@
           <t>Das 171 frotas programadas para as semanas 40/41 11% ficou sem justificativa e 23,4% ficou sem apontamento.</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Feito
+</t>
+        </is>
+      </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -790,8 +816,16 @@
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr">
         <is>
           <t>Causa: falta conscientização do colaborador para realizar a os apontamentos</t>
@@ -802,10 +836,15 @@
           <t>Das 171 frotas programadas para as semanas 40/41 11% ficou sem justificativa e 23,4% ficou sem apontamento.</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Feito
+</t>
+        </is>
+      </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1709,7 +1748,7 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Planejada</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">

</xml_diff>

<commit_message>
Auto-atualização RTA - 24/10/2026 12:02
</commit_message>
<xml_diff>
--- a/downloads/RTA_Dados.xlsx
+++ b/downloads/RTA_Dados.xlsx
@@ -529,7 +529,7 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>Atrasada</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -1748,7 +1748,7 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>Atrasada</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">

</xml_diff>

<commit_message>
Auto-atualização RTA - 26/10/2026 12:02
</commit_message>
<xml_diff>
--- a/downloads/RTA_Dados.xlsx
+++ b/downloads/RTA_Dados.xlsx
@@ -9552,8 +9552,16 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="G149" t="inlineStr"/>
-      <c r="H149" t="inlineStr"/>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
       <c r="I149" t="inlineStr">
         <is>
           <t>Causa: Falta de dados pro colhedora offline</t>
@@ -9564,10 +9572,14 @@
           <t>entre os dias 26 a 31/05 não atingiu a meta de 76% eficiência operacional</t>
         </is>
       </c>
-      <c r="K149" t="inlineStr"/>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Starlink instalada na frente 23 </t>
+        </is>
+      </c>
       <c r="L149" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M149" t="inlineStr">

</xml_diff>

<commit_message>
Auto-atualização RTA - 27/10/2026 12:02
</commit_message>
<xml_diff>
--- a/downloads/RTA_Dados.xlsx
+++ b/downloads/RTA_Dados.xlsx
@@ -514,8 +514,16 @@
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
           <t>Causa: Os operadores no momento não sentiram necessidade de cumprir o padrão</t>
@@ -526,10 +534,15 @@
           <t>No dia 12/10/2026 o pulmão ficou abaixo da limite inferior por 4 horas seguidas, aconteceu no turno C as 4:00 da manhã, estavamos com a moagem elevada e várias ocorrências no campo, disponibilidade, terceiro com baixa entrega, frente mudando de área, na análise faltou o senso de redução da moagem com antecedência.</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Concluído 
+[fig:vfs:3361]</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -13553,8 +13566,16 @@
           <t>2026-05-14</t>
         </is>
       </c>
-      <c r="G206" t="inlineStr"/>
-      <c r="H206" t="inlineStr"/>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
       <c r="I206" t="inlineStr">
         <is>
           <t>Causa: não fizemos manutenção por motivo de falta peças</t>
@@ -13569,7 +13590,7 @@
       <c r="K206" t="inlineStr"/>
       <c r="L206" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M206" t="inlineStr">
@@ -13609,8 +13630,16 @@
           <t>2026-05-15</t>
         </is>
       </c>
-      <c r="G207" t="inlineStr"/>
-      <c r="H207" t="inlineStr"/>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
       <c r="I207" t="inlineStr">
         <is>
           <t>Causa: não fizemos manutenção por motivo de falta peças</t>
@@ -13625,7 +13654,7 @@
       <c r="K207" t="inlineStr"/>
       <c r="L207" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M207" t="inlineStr">

</xml_diff>

<commit_message>
Auto-atualização RTA - 27/10/2026 15:42
</commit_message>
<xml_diff>
--- a/downloads/RTA_Dados.xlsx
+++ b/downloads/RTA_Dados.xlsx
@@ -13028,8 +13028,16 @@
           <t>2026-08-11</t>
         </is>
       </c>
-      <c r="G198" t="inlineStr"/>
-      <c r="H198" t="inlineStr"/>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
       <c r="I198" t="inlineStr">
         <is>
           <t>Causa: Válvula danificada da caixa 04</t>
@@ -13049,10 +13057,14 @@
 [fig:vfs:2481]</t>
         </is>
       </c>
-      <c r="K198" t="inlineStr"/>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t>INSTALADO VALVULAS PARA CONFERENCIA DE POSSIVEIS VAZAMENTOS DE CALDO EM VALVULAS DANDO PASSAGEM.</t>
+        </is>
+      </c>
       <c r="L198" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M198" t="inlineStr">

</xml_diff>

<commit_message>
Auto-atualização RTA - 29/10/2026 12:57
</commit_message>
<xml_diff>
--- a/downloads/RTA_Dados.xlsx
+++ b/downloads/RTA_Dados.xlsx
@@ -2934,8 +2934,16 @@
           <t>2027-09-30</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr"/>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="I43" t="inlineStr">
         <is>
           <t>Causa: Lubrificante Inadequado</t>
@@ -2947,10 +2955,14 @@
 Após algumas horas de operação, o líder do setor identificou ruído anormal no equipamento e solicitou a presença do mecânico P26 para avaliação. Durante a intervenção, o mecânico realizou a aplicação de graxa no mancal. Logo após a lubrificação, o equipamento apresentou emissão de fumaça e elevação acentuada da temperatura do mancal.</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr"/>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Indicação da graxa correta e suas respectivas quantidades na lubrificação dos mancais dos ventiladores e exaustores das caldeiras.</t>
+        </is>
+      </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>Planejada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -3046,7 +3058,11 @@
           <t>2027-04-01</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr"/>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
       <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr">
         <is>
@@ -3059,10 +3075,14 @@
 Após algumas horas de operação, o líder do setor identificou ruído anormal no equipamento e solicitou a presença do mecânico P26 para avaliação. Durante a intervenção, o mecânico realizou a aplicação de graxa no mancal. Logo após a lubrificação, o equipamento apresentou emissão de fumaça e elevação acentuada da temperatura do mancal.</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr"/>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Treinamento em Lubrificação Básica realizado para os Lubrificadores.</t>
+        </is>
+      </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>Planejada</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
@@ -3102,8 +3122,16 @@
           <t>2026-10-31</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
       <c r="I46" t="inlineStr">
         <is>
           <t>Causa: Plano de lubrificação mancais ventiladores/exaustores incorreto</t>
@@ -3115,10 +3143,14 @@
 Após algumas horas de operação, o líder do setor identificou ruído anormal no equipamento e solicitou a presença do mecânico P26 para avaliação. Durante a intervenção, o mecânico realizou a aplicação de graxa no mancal. Logo após a lubrificação, o equipamento apresentou emissão de fumaça e elevação acentuada da temperatura do mancal.</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr"/>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Feito treinamento das novas quantidades de graxas na lubrificação dos ventiladores e exaustores.</t>
+        </is>
+      </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>Planejada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
@@ -3158,8 +3190,16 @@
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="I47" t="inlineStr">
         <is>
           <t>Causa: Intervalo de medição alto</t>
@@ -3171,10 +3211,14 @@
 Após algumas horas de operação, o líder do setor identificou ruído anormal no equipamento e solicitou a presença do mecânico P26 para avaliação. Durante a intervenção, o mecânico realizou a aplicação de graxa no mancal. Logo após a lubrificação, o equipamento apresentou emissão de fumaça e elevação acentuada da temperatura do mancal.</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr"/>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Realizada a adequação do intervalo de relubrificação dos mancais dos ventiladores e exaustores. Procedimento in loco.</t>
+        </is>
+      </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
@@ -4915,8 +4959,16 @@
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr"/>
-      <c r="H75" t="inlineStr"/>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
       <c r="I75" t="inlineStr">
         <is>
           <t>Causa: Lubrificante inadequado para aplicação (impurezas no lubrificante)</t>
@@ -4927,10 +4979,14 @@
           <t>Identificado ponto incandescente na intermediária 1, ao inspecionar rolamento mancal lado acoplado estava quebrado em alinhamento entre especialista do turno e coordenador de manutenção se decidiu parar a Moenda e desmontar o equipamento</t>
         </is>
       </c>
-      <c r="K75" t="inlineStr"/>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>Feito. Desde o dia do incidente, a lubrificação passou ser a com a graxa de sulfonato de cálcio.</t>
+        </is>
+      </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M75" t="inlineStr">
@@ -4970,8 +5026,16 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr"/>
-      <c r="H76" t="inlineStr"/>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
       <c r="I76" t="inlineStr">
         <is>
           <t>Causa: Falha no plano de lubrificação</t>
@@ -4982,10 +5046,14 @@
           <t>Identificado ponto incandescente na intermediária 1, ao inspecionar rolamento mancal lado acoplado estava quebrado em alinhamento entre especialista do turno e coordenador de manutenção se decidiu parar a Moenda e desmontar o equipamento</t>
         </is>
       </c>
-      <c r="K76" t="inlineStr"/>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Realizado o acompanhamento e desvios apontados em e-mail. </t>
+        </is>
+      </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M76" t="inlineStr">
@@ -5025,8 +5093,16 @@
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="G77" t="inlineStr"/>
-      <c r="H77" t="inlineStr"/>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
       <c r="I77" t="inlineStr">
         <is>
           <t>Causa: Labirinto do mancal fixado com abraçadeira</t>
@@ -5037,10 +5113,14 @@
           <t>Identificado ponto incandescente na intermediária 1, ao inspecionar rolamento mancal lado acoplado estava quebrado em alinhamento entre especialista do turno e coordenador de manutenção se decidiu parar a Moenda e desmontar o equipamento</t>
         </is>
       </c>
-      <c r="K77" t="inlineStr"/>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>Realizado acompanhamento das rotas de lubrificação e apontado melhorias. Instruções verbais no momento da aplicação junto aos Lubrificadores.</t>
+        </is>
+      </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M77" t="inlineStr">
@@ -11936,8 +12016,16 @@
           <t>2026-06-12</t>
         </is>
       </c>
-      <c r="G183" t="inlineStr"/>
-      <c r="H183" t="inlineStr"/>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
       <c r="I183" t="inlineStr">
         <is>
           <t>Causa: Bomba reserva não atende</t>
@@ -11958,10 +12046,14 @@
 [fig:vfs:2623]</t>
         </is>
       </c>
-      <c r="K183" t="inlineStr"/>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>A pré- ordem foi aberta, e atualmente estamos usando um conjunto de dispersante e antiespumante que atende o processo.</t>
+        </is>
+      </c>
       <c r="L183" t="inlineStr">
         <is>
-          <t>Atrasada</t>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="M183" t="inlineStr">

</xml_diff>

<commit_message>
Auto-atualização RTA - 30/10/2026 16:30
</commit_message>
<xml_diff>
--- a/downloads/RTA_Dados.xlsx
+++ b/downloads/RTA_Dados.xlsx
@@ -531,7 +531,7 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Planejada</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -588,7 +588,7 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Planejada</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -1474,7 +1474,7 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Planejada</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2661,7 +2661,7 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Planejada</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -4974,7 +4974,7 @@
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
-          <t>Planejada</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="M75" t="inlineStr">

</xml_diff>

<commit_message>
Auto-atualização RTA - 31/10/2026 12:02
</commit_message>
<xml_diff>
--- a/downloads/RTA_Dados.xlsx
+++ b/downloads/RTA_Dados.xlsx
@@ -531,7 +531,7 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>Atrasada</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -588,7 +588,7 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>Atrasada</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -881,7 +881,7 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Planejada</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1474,7 +1474,7 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>Atrasada</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2661,7 +2661,7 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>Atrasada</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -4974,7 +4974,7 @@
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>Atrasada</t>
         </is>
       </c>
       <c r="M75" t="inlineStr">

</xml_diff>